<commit_message>
#172 JLCPCB BOM and Centroid Completed
</commit_message>
<xml_diff>
--- a/BOM/TDS_Meter/eSpark_BOM_TDS_Meter.xlsx
+++ b/BOM/TDS_Meter/eSpark_BOM_TDS_Meter.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\OliverStanton-WaterMonitor\BOM\TDS_Meter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\OliverStanton-WaterMonitor\BOM\TDS_Meter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D635BE-3CE8-4DFC-BC17-1679EDC892BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -279,7 +278,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -747,7 +746,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -963,6 +962,15 @@
     <xf numFmtId="0" fontId="23" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1304,7 +1312,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:S19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1635,51 +1643,51 @@
       <c r="C11" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="50" t="s">
+      <c r="D11" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="51" t="s">
+      <c r="E11" s="79" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="50" t="s">
+      <c r="F11" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="51" t="s">
+      <c r="G11" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="H11" s="50" t="s">
+      <c r="H11" s="78" t="s">
         <v>60</v>
       </c>
-      <c r="I11" s="51" t="s">
+      <c r="I11" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="J11" s="50" t="s">
+      <c r="J11" s="78" t="s">
         <v>60</v>
       </c>
-      <c r="K11" s="50" t="s">
+      <c r="K11" s="78" t="s">
         <v>60</v>
       </c>
-      <c r="L11" s="51">
+      <c r="L11" s="79">
         <v>2</v>
       </c>
-      <c r="M11" s="50">
+      <c r="M11" s="78">
         <f t="shared" ref="M11:M17" si="1">L11*5</f>
         <v>10</v>
       </c>
-      <c r="N11" s="51" t="s">
+      <c r="N11" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="O11" s="50" t="s">
+      <c r="O11" s="78" t="s">
         <v>60</v>
       </c>
-      <c r="P11" s="51" t="s">
+      <c r="P11" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="Q11" s="54" t="s">
+      <c r="Q11" s="80" t="s">
         <v>60</v>
       </c>
-      <c r="R11" s="51"/>
-      <c r="S11" s="50"/>
+      <c r="R11" s="79"/>
+      <c r="S11" s="78"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -2078,13 +2086,13 @@
     <mergeCell ref="N19:P19"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O12" r:id="rId1" xr:uid="{977987ED-9FE0-47B0-AE46-5E17A351811B}"/>
-    <hyperlink ref="O13" r:id="rId2" xr:uid="{906AFE4B-000D-4BD8-84A7-A8A2395DE921}"/>
-    <hyperlink ref="O10" r:id="rId3" xr:uid="{A56A9E6B-703A-4BF6-8798-9FD31E2A2303}"/>
-    <hyperlink ref="O14" r:id="rId4" xr:uid="{5B97FE88-D43B-436B-AB56-8FA9D5EEE38F}"/>
-    <hyperlink ref="O15" r:id="rId5" xr:uid="{ACC32550-621C-44EA-AC13-21D551231C73}"/>
-    <hyperlink ref="O16" r:id="rId6" xr:uid="{7CD3887C-D4F2-4263-96AB-59D006D9F851}"/>
-    <hyperlink ref="O17" r:id="rId7" xr:uid="{FE696CC9-9A60-4A3E-A77B-33D07A936CD4}"/>
+    <hyperlink ref="O12" r:id="rId1"/>
+    <hyperlink ref="O13" r:id="rId2"/>
+    <hyperlink ref="O10" r:id="rId3"/>
+    <hyperlink ref="O14" r:id="rId4"/>
+    <hyperlink ref="O15" r:id="rId5"/>
+    <hyperlink ref="O16" r:id="rId6"/>
+    <hyperlink ref="O17" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>

</xml_diff>